<commit_message>
Actualizacao dados de poupancas e os graficos de visualizacao
</commit_message>
<xml_diff>
--- a/Geral_Poupanca.xlsx
+++ b/Geral_Poupanca.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>220</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -484,17 +484,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3840</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nada</t>
+          <t>NICANE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -514,17 +509,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3918786000010250014</t>
+          <t>3918786000010250008</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>MUDANCA DE VIDA</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>MUDANCA DE VIDA</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -534,12 +529,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>23000</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -549,42 +544,1727 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>3 Sessão</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2490</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>18655</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>3918786000010254032</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3780</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>13-May-2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>3918786000010250008</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>MUDANCA DE VIDA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>MUDANCA DE VIDA</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>22900</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2 Sessão</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>18145</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>3918786000010254030</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3700</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>06-May-2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>3918786000010250008</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>MUDANCA DE VIDA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>MUDANCA DE VIDA</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>21900</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>1 Sessão</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>3918786000010252002</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>17585</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>3918786000010254028</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>340</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3060</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>20-May-2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>3918786000010250010</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ORUWERA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ORUWERA</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>18200</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2 Sessão</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1220</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>14425</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>3918786000010254026</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2980</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>13-May-2026</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>3918786000010250010</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ORUWERA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ORUWERA</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>18200</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1 Sessão</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>580</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>13845</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>3918786000010254024</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>340</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2640</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>20-May-2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>3918786000010250012</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>UNIAO FAZ A FORCA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>UNIAO FAZ A FORCA</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>17000</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>3 Sessão</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>12645</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>3918786000010254022</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2430</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>13-May-2026</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>3918786000010250012</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>UNIAO FAZ A FORCA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>UNIAO FAZ A FORCA</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>15200</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2 Sessão</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1080</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>11565</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>3918786000010254020</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2300</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>06-May-2026</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>3918786000010250012</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>UNIAO FAZ A FORCA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UNIAO FAZ A FORCA</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>15200</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1 Sessão</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>760</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>10805</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>3918786000010254018</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>14-May-2026</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>12200</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>7 Sessão</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1240</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>9565</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>3918786000010254016</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>410</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1560</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>07-May-2026</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>9000</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>6 Sessão</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>3200</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>8065</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>3918786000010254014</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1240</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>30-Apr-2026</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>5 Sessão</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1650</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>6415</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>3918786000010254012</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>890</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>23-Apr-2026</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>4000</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>4 Sessão</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>4455</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>3918786000010254010</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>640</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>16-Apr-2026</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>3 Sessão</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>3405</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>3918786000010254008</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compra de 3 pratos </t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>09-Apr-2026</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>2 Sessão</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1700</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>1705</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>3918786000010254006</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>02-Apr-2026</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1 Sessão</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>3918786000010254004</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>14-May-2026</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>3918786000010250004</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>WIKHALIHERA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>WIKHALIHERA</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1 Sessão</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>3918786000010254002</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -849,13 +2529,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20A2AD10-923F-454F-AAFD-DE68639D7C28}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{392BE2BC-BDEB-4D6C-8D3E-D2B97F97C516}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{414B9C67-B917-4FA4-8CD9-E2AC262CC649}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F97496F9-18D6-4E56-BB56-173E0B9F2D8E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D21B4C37-C9CF-46AF-BB5D-441FD219F47D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BED42028-C3EA-4283-893B-3D3F275E45C0}"/>
 </file>
</xml_diff>

<commit_message>
Observe da pagina pou
</commit_message>
<xml_diff>
--- a/Geral_Poupanca.xlsx
+++ b/Geral_Poupanca.xlsx
@@ -7852,4 +7852,271 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
+    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A8B9A46-65C0-428A-A514-29B3552FF2BC}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C934F88-56F9-47B7-A625-90461FC9B0A1}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9985BED6-620A-4FA7-B1FB-960AF24CCEBC}"/>
 </file>
</xml_diff>